<commit_message>
ALPHADHABI: reweight lenses 55/15/15/15 (from 45/15/25/15) — look-through cut 25%→15% on external-audit double-count flag, freed 10pts to the SOTP anchor. Weighted central 7.30→7.13 (spot -13% vs -11%); band 5.95-8.63. Rebased onto EAND publish.
</commit_message>
<xml_diff>
--- a/files/ALPHADHABI_Valuation_Model_10-07-2026_public.xlsx
+++ b/files/ALPHADHABI_Valuation_Model_10-07-2026_public.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">Weighted central (12-mo, risk-adjusted)</t>
   </si>
   <si>
-    <t xml:space="preserve">AED 7.30  (range 6.08–8.82)</t>
+    <t xml:space="preserve">AED 7.13  (range 5.95–8.63)</t>
   </si>
   <si>
     <t xml:space="preserve">60-day MC band (5–95%)</t>
@@ -734,7 +734,7 @@
     <t xml:space="preserve">high</t>
   </si>
   <si>
-    <t xml:space="preserve">Published weights 45/15/25/15</t>
+    <t xml:space="preserve">Published weights 55/15/15/15</t>
   </si>
   <si>
     <t xml:space="preserve">Monte Carlo engine — v3 carry-anchored YZ-HAR-t, AE provisional fit</t>
@@ -1412,7 +1412,7 @@
     <t xml:space="preserve">Durable ceasefire + Fed cutting → ~7.4; month-plus Hormuz closure or accelerated Pillar-Two top-ups → ~6.4</t>
   </si>
   <si>
-    <t xml:space="preserve">Panel span AED 6.3–7.0 vs weighted central 7.30 — all three land below spot 8.22.</t>
+    <t xml:space="preserve">Panel span AED 6.3–7.0 vs weighted central 7.13 — all three land below spot 8.22.</t>
   </si>
   <si>
     <t xml:space="preserve">Per-Share &amp; Ratios — the standardized dashboard</t>
@@ -6369,13 +6369,13 @@
         <v>232</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>6.08</v>
+        <v>5.95</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>7.3</v>
+        <v>7.13</v>
       </c>
       <c r="D23" s="9" t="n">
-        <v>8.82</v>
+        <v>8.63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>